<commit_message>
ingesta: Teoria Relacionada acepta apuntes directos; actualizar content/
Teoria Relacionada puede nombrar un tema del programa o directamente un
apunte (.pdf/.md); se avisa si el archivo no existe en content/apuntes.
Planilla de prácticas corregida (prácticas 4 y Extra) y apuntes renombrados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Prácticas Bases de Datos.xlsx
+++ b/content/Prácticas Bases de Datos.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{693B27A7-F451-445F-AC59-1D201394AF93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E78B71F3-A9A3-41E8-A017-A86CFC0EF96C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="213">
   <si>
     <t>NumeroPractica</t>
   </si>
@@ -68,13 +68,22 @@
 4. En Español de Argentina la manera correcta de referirse al JOIN es Junta. Al LEFT OUTER JOIN, junta izquierda. A la unión de conjuntos UNION, y a la unión de multiconjuntos UNION ALL. No confundir unión con junta.</t>
   </si>
   <si>
-    <t>["Modelo Relacional","Algebra relacional: Operaciones, Práctica","Lenguajes relacionalmente completos"]</t>
+    <t>["001 - Taller#3 - Apunte - Lenguajes relacionales.pdf","009 - Taller #8 - Visuals - De Algebra Relacional a SQL.pdf"]</t>
   </si>
   <si>
     <t>Algebra Relacional - SQL - Practica 2</t>
   </si>
   <si>
     <t>Algebra Relacional - SQL - Practica 3</t>
+  </si>
+  <si>
+    <t>Algebra Relacional - SQL - Practica 4</t>
+  </si>
+  <si>
+    <t>Extra</t>
+  </si>
+  <si>
+    <t>Algebra Relacional - SQL - Practica Extra</t>
   </si>
   <si>
     <t>Tip</t>
@@ -450,9 +459,6 @@
 Partes.nombre y se calcula el promedio del costo."]</t>
   </si>
   <si>
-    <t>Extra</t>
-  </si>
-  <si>
     <t>Dadas las siguientes relaciones:
 SOCIO (aficionado, videoclub)
 GUSTA (aficionado, pelicula)
@@ -498,6 +504,101 @@
   </si>
   <si>
     <t>["Se obtiene el conjunto de aficionados que, siendo socios, tienen en la videoteca del videoclub alguna película que también les gusta (la unión de SOCIO, VIDEOTECA y GUSTA con los criterios indicados). Luego se resta ese conjunto del conjunto de todos los aficionados (extraído de GUSTA). El resultado es el conjunto de aficionados que no son socios de ningún videoclub que disponga de alguna película de su gusto."]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolver en Algebra Relacional y SQL para el siguiente esquema: CREATE TABLE oficina ( 
+  codigo_oficina VARCHAR(10) NOT NULL, 
+  ciudad VARCHAR(30) NOT NULL, 
+  pais VARCHAR(50) NOT NULL, 
+  region VARCHAR(50) DEFAULT NULL, 
+  codigo_postal VARCHAR(10) NOT NULL, 
+  telefono VARCHAR(20) NOT NULL, 
+  linea_direccion1 VARCHAR(50) NOT NULL, 
+  linea_direccion2 VARCHAR(50) DEFAULT NULL, 
+  PRIMARY KEY (codigo_oficina) 
+); 
+CREATE TABLE empleado ( 
+  codigo_empleado INTEGER NOT NULL, 
+  nombre VARCHAR(50) NOT NULL, 
+  apellido1 VARCHAR(50) NOT NULL, 
+  apellido2 VARCHAR(50) DEFAULT NULL, 
+  extension VARCHAR(10) NOT NULL, 
+  email VARCHAR(100) NOT NULL, 
+  codigo_oficina VARCHAR(10) NOT NULL, 
+  codigo_jefe INTEGER DEFAULT NULL, 
+  puesto VARCHAR(50) DEFAULT NULL, 
+  PRIMARY KEY (codigo_empleado), 
+  FOREIGN KEY (codigo_oficina) REFERENCES oficina (codigo_oficina), 
+  FOREIGN KEY (codigo_jefe) REFERENCES empleado (codigo_empleado) 
+); 
+CREATE TABLE gama_producto ( 
+  gama VARCHAR(50) NOT NULL, 
+  descripcion_texto TEXT, 
+  descripcion_html TEXT, 
+  imagen VARCHAR(256), 
+  PRIMARY KEY (gama) 
+); 
+CREATE TABLE cliente ( 
+  codigo_cliente INTEGER NOT NULL, 
+  nombre_cliente VARCHAR(50) NOT NULL, 
+  nombre_contacto VARCHAR(30) DEFAULT NULL, 
+  apellido_contacto VARCHAR(30) DEFAULT NULL, 
+  telefono VARCHAR(15) NOT NULL, 
+  fax VARCHAR(15) NOT NULL, 
+  linea_direccion1 VARCHAR(50) NOT NULL, 
+  linea_direccion2 VARCHAR(50) DEFAULT NULL, 
+  ciudad VARCHAR(50) NOT NULL, 
+  region VARCHAR(50) DEFAULT NULL, 
+  pais VARCHAR(50) DEFAULT NULL, 
+  codigo_postal VARCHAR(10) DEFAULT NULL, 
+  codigo_empleado_rep_ventas INTEGER DEFAULT NULL, 
+  limite_credito NUMERIC(15,2) DEFAULT NULL, 
+  PRIMARY KEY (codigo_cliente), 
+  FOREIGN KEY (codigo_empleado_rep_ventas) REFERENCES empleado (codigo_empleado) 
+); 
+CREATE TABLE pedido ( 
+  codigo_pedido INTEGER NOT NULL, 
+  fecha_pedido date NOT NULL, 
+  fecha_esperada date NOT NULL, 
+  fecha_entrega date DEFAULT NULL, 
+  estado VARCHAR(15) NOT NULL, 
+  comentarios TEXT, 
+  codigo_cliente INTEGER NOT NULL, 
+  PRIMARY KEY (codigo_pedido), 
+  FOREIGN KEY (codigo_cliente) REFERENCES cliente (codigo_cliente) 
+); 
+CREATE TABLE producto ( 
+  codigo_producto VARCHAR(15) NOT NULL, 
+  nombre VARCHAR(70) NOT NULL, 
+  gama VARCHAR(50) NOT NULL, 
+  dimensiones VARCHAR(25) NULL, 
+  proveedor VARCHAR(50) DEFAULT NULL, 
+  descripcion text NULL, 
+  cantidad_en_stock SMALLINT NOT NULL, 
+  precio_venta NUMERIC(15,2) NOT NULL, 
+  precio_proveedor NUMERIC(15,2) DEFAULT NULL, 
+  PRIMARY KEY (codigo_producto), 
+  FOREIGN KEY (gama) REFERENCES gama_producto (gama) 
+); 
+CREATE TABLE detalle_pedido ( 
+  codigo_pedido INTEGER NOT NULL, 
+  codigo_producto VARCHAR(15) NOT NULL, 
+  cantidad INTEGER NOT NULL, 
+  precio_unidad NUMERIC(15,2) NOT NULL, 
+  numero_linea SMALLINT NOT NULL, 
+  PRIMARY KEY (codigo_pedido, codigo_producto), 
+  FOREIGN KEY (codigo_pedido) REFERENCES pedido (codigo_pedido), 
+  FOREIGN KEY (codigo_producto) REFERENCES producto (codigo_producto) 
+); 
+CREATE TABLE pago ( 
+  codigo_cliente INTEGER NOT NULL, 
+  forma_pago VARCHAR(40) NOT NULL, 
+  id_transaccion VARCHAR(50) NOT NULL, 
+  fecha_pago date NOT NULL, 
+  total NUMERIC(15,2) NOT NULL, 
+  PRIMARY KEY (codigo_cliente, id_transaccion), 
+  FOREIGN KEY (codigo_cliente) REFERENCES cliente (codigo_cliente) 
+); </t>
   </si>
   <si>
     <t>1. Devuelva un listado con el código de oficina y la ciudad donde hay oficinas.</t>
@@ -1110,7 +1211,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE89438-0AA0-4FDB-B7D9-02DE1265A35C}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
@@ -1197,6 +1298,46 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="144.75">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="144.75">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1219,7 +1360,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16.5" customHeight="1">
@@ -1227,7 +1368,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="29.25">
@@ -1235,7 +1376,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="43.5">
@@ -1243,7 +1384,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1251,7 +1392,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="29.25">
@@ -1259,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="43.5">
@@ -1267,7 +1408,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="43.5">
@@ -1275,7 +1416,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="43.5">
@@ -1283,7 +1424,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1291,7 +1432,7 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1315,22 +1456,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="105.75" customHeight="1">
@@ -1338,16 +1479,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1355,22 +1496,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.5">
@@ -1378,22 +1519,22 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="43.5">
@@ -1401,22 +1542,22 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="109.5" customHeight="1">
@@ -1424,22 +1565,22 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.5">
@@ -1447,22 +1588,22 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="29.25">
@@ -1470,22 +1611,22 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="90">
@@ -1493,19 +1634,19 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="75.75">
@@ -1513,19 +1654,19 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="45">
@@ -1533,19 +1674,19 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="170.25" customHeight="1">
@@ -1553,13 +1694,13 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="45">
@@ -1567,19 +1708,19 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="43.5">
@@ -1587,19 +1728,19 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="136.5" customHeight="1">
@@ -1607,13 +1748,13 @@
         <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="46.5">
@@ -1621,19 +1762,19 @@
         <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="46.5">
@@ -1641,22 +1782,22 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="48">
@@ -1664,19 +1805,19 @@
         <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="122.25">
@@ -1684,22 +1825,22 @@
         <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30.75">
@@ -1707,19 +1848,19 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="132">
@@ -1727,19 +1868,19 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="177">
@@ -1747,22 +1888,22 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G22" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="104.25">
@@ -1770,22 +1911,22 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30.75">
@@ -1793,22 +1934,22 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G24" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="147.75">
@@ -1816,19 +1957,19 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="63">
@@ -1836,19 +1977,19 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="189.75">
@@ -1856,19 +1997,19 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="64.5">
@@ -1876,22 +2017,22 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G28" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="60.75">
@@ -1899,19 +2040,19 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="102.75">
@@ -1919,22 +2060,22 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="147.75">
@@ -1942,19 +2083,19 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="101.25">
@@ -1962,136 +2103,147 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C32">
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="124.5" customHeight="1">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C34">
         <v>1</v>
       </c>
       <c r="D34" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="30.75">
       <c r="A35" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="46.5">
       <c r="A36" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C36">
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G36" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="281.25">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>14</v>
       </c>
       <c r="B37" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="409.6">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
         <v>32</v>
       </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-      <c r="D37" t="s">
-        <v>45</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="E38" s="1"/>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39">
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -2100,7 +2252,7 @@
         <v>1</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2108,7 +2260,7 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -2117,7 +2269,7 @@
         <v>2</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="29.25">
@@ -2125,7 +2277,7 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -2134,7 +2286,7 @@
         <v>3</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="29.25">
@@ -2142,7 +2294,7 @@
         <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -2151,7 +2303,7 @@
         <v>4</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="29.25">
@@ -2159,7 +2311,7 @@
         <v>4</v>
       </c>
       <c r="B43" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2168,7 +2320,7 @@
         <v>5</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -2176,7 +2328,7 @@
         <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -2185,7 +2337,7 @@
         <v>6</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="29.25">
@@ -2193,7 +2345,7 @@
         <v>4</v>
       </c>
       <c r="B45" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2202,7 +2354,7 @@
         <v>7</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="43.5">
@@ -2210,7 +2362,7 @@
         <v>4</v>
       </c>
       <c r="B46" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -2219,7 +2371,7 @@
         <v>8</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="29.25">
@@ -2227,7 +2379,7 @@
         <v>4</v>
       </c>
       <c r="B47" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -2236,7 +2388,7 @@
         <v>9</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="43.5">
@@ -2244,7 +2396,7 @@
         <v>4</v>
       </c>
       <c r="B48" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -2253,7 +2405,7 @@
         <v>10</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="29.25">
@@ -2261,7 +2413,7 @@
         <v>4</v>
       </c>
       <c r="B49" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -2270,7 +2422,7 @@
         <v>11</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="29.25">
@@ -2278,7 +2430,7 @@
         <v>4</v>
       </c>
       <c r="B50" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -2287,7 +2439,7 @@
         <v>12</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="29.25">
@@ -2295,7 +2447,7 @@
         <v>4</v>
       </c>
       <c r="B51" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -2304,7 +2456,7 @@
         <v>13</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="57.75">
@@ -2312,7 +2464,7 @@
         <v>4</v>
       </c>
       <c r="B52" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2321,7 +2473,7 @@
         <v>14</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="29.25">
@@ -2329,7 +2481,7 @@
         <v>4</v>
       </c>
       <c r="B53" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -2338,7 +2490,7 @@
         <v>15</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="29.25">
@@ -2346,7 +2498,7 @@
         <v>4</v>
       </c>
       <c r="B54" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -2355,7 +2507,7 @@
         <v>16</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="29.25">
@@ -2363,7 +2515,7 @@
         <v>4</v>
       </c>
       <c r="B55" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -2372,7 +2524,7 @@
         <v>17</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="29.25">
@@ -2380,7 +2532,7 @@
         <v>4</v>
       </c>
       <c r="B56" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -2389,7 +2541,7 @@
         <v>18</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="29.25">
@@ -2397,7 +2549,7 @@
         <v>4</v>
       </c>
       <c r="B57" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -2406,7 +2558,7 @@
         <v>19</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="29.25">
@@ -2414,7 +2566,7 @@
         <v>4</v>
       </c>
       <c r="B58" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2423,7 +2575,7 @@
         <v>20</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="29.25">
@@ -2431,7 +2583,7 @@
         <v>4</v>
       </c>
       <c r="B59" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -2440,7 +2592,7 @@
         <v>21</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="29.25">
@@ -2448,7 +2600,7 @@
         <v>4</v>
       </c>
       <c r="B60" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -2457,7 +2609,7 @@
         <v>22</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="29.25">
@@ -2465,7 +2617,7 @@
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -2474,7 +2626,7 @@
         <v>23</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="43.5">
@@ -2482,7 +2634,7 @@
         <v>4</v>
       </c>
       <c r="B62" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -2491,7 +2643,7 @@
         <v>24</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="43.5">
@@ -2499,7 +2651,7 @@
         <v>4</v>
       </c>
       <c r="B63" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -2508,7 +2660,7 @@
         <v>25</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="29.25">
@@ -2516,7 +2668,7 @@
         <v>4</v>
       </c>
       <c r="B64" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C64">
         <v>1</v>
@@ -2525,7 +2677,7 @@
         <v>26</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="29.25">
@@ -2533,7 +2685,7 @@
         <v>4</v>
       </c>
       <c r="B65" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -2542,7 +2694,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -2550,7 +2702,7 @@
         <v>4</v>
       </c>
       <c r="B66" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C66">
         <v>1</v>
@@ -2559,7 +2711,7 @@
         <v>28</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -2567,7 +2719,7 @@
         <v>4</v>
       </c>
       <c r="B67" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -2576,7 +2728,7 @@
         <v>29</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -2584,7 +2736,7 @@
         <v>4</v>
       </c>
       <c r="B68" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -2593,7 +2745,7 @@
         <v>30</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="29.25">
@@ -2601,7 +2753,7 @@
         <v>4</v>
       </c>
       <c r="B69" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -2610,7 +2762,7 @@
         <v>31</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="29.25">
@@ -2618,7 +2770,7 @@
         <v>4</v>
       </c>
       <c r="B70" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -2627,7 +2779,7 @@
         <v>32</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -2635,7 +2787,7 @@
         <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -2644,7 +2796,7 @@
         <v>33</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -2652,7 +2804,7 @@
         <v>4</v>
       </c>
       <c r="B72" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C72">
         <v>1</v>
@@ -2661,7 +2813,7 @@
         <v>34</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="29.25">
@@ -2669,7 +2821,7 @@
         <v>4</v>
       </c>
       <c r="B73" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C73">
         <v>1</v>
@@ -2678,7 +2830,7 @@
         <v>35</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="29.25">
@@ -2686,7 +2838,7 @@
         <v>4</v>
       </c>
       <c r="B74" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -2695,7 +2847,7 @@
         <v>36</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="29.25">
@@ -2703,7 +2855,7 @@
         <v>4</v>
       </c>
       <c r="B75" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -2712,7 +2864,7 @@
         <v>37</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="29.25">
@@ -2720,7 +2872,7 @@
         <v>4</v>
       </c>
       <c r="B76" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C76">
         <v>1</v>
@@ -2729,7 +2881,7 @@
         <v>38</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="29.25">
@@ -2737,7 +2889,7 @@
         <v>4</v>
       </c>
       <c r="B77" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -2746,7 +2898,7 @@
         <v>39</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="29.25">
@@ -2754,7 +2906,7 @@
         <v>4</v>
       </c>
       <c r="B78" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -2763,7 +2915,7 @@
         <v>40</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="43.5">
@@ -2771,7 +2923,7 @@
         <v>4</v>
       </c>
       <c r="B79" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -2780,7 +2932,7 @@
         <v>41</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="72.75">
@@ -2788,7 +2940,7 @@
         <v>4</v>
       </c>
       <c r="B80" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -2797,7 +2949,7 @@
         <v>42</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="72.75">
@@ -2805,7 +2957,7 @@
         <v>4</v>
       </c>
       <c r="B81" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -2814,7 +2966,7 @@
         <v>43</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="87">
@@ -2822,7 +2974,7 @@
         <v>4</v>
       </c>
       <c r="B82" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C82">
         <v>1</v>
@@ -2831,7 +2983,7 @@
         <v>44</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="43.5">
@@ -2839,7 +2991,7 @@
         <v>4</v>
       </c>
       <c r="B83" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -2848,7 +3000,7 @@
         <v>45</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="29.25">
@@ -2856,7 +3008,7 @@
         <v>4</v>
       </c>
       <c r="B84" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C84">
         <v>1</v>
@@ -2865,7 +3017,7 @@
         <v>46</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -2873,7 +3025,7 @@
         <v>4</v>
       </c>
       <c r="B85" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C85">
         <v>1</v>
@@ -2882,7 +3034,7 @@
         <v>47</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -2890,7 +3042,7 @@
         <v>4</v>
       </c>
       <c r="B86" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C86">
         <v>1</v>
@@ -2899,7 +3051,7 @@
         <v>48</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="57.75">
@@ -2907,7 +3059,7 @@
         <v>4</v>
       </c>
       <c r="B87" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C87">
         <v>1</v>
@@ -2916,7 +3068,7 @@
         <v>49</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="29.25">
@@ -2924,7 +3076,7 @@
         <v>4</v>
       </c>
       <c r="B88" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C88">
         <v>1</v>
@@ -2933,7 +3085,7 @@
         <v>50</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -2941,7 +3093,7 @@
         <v>4</v>
       </c>
       <c r="B89" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C89">
         <v>1</v>
@@ -2950,7 +3102,7 @@
         <v>51</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -2958,7 +3110,7 @@
         <v>4</v>
       </c>
       <c r="B90" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C90">
         <v>1</v>
@@ -2967,7 +3119,7 @@
         <v>52</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="29.25">
@@ -2975,7 +3127,7 @@
         <v>4</v>
       </c>
       <c r="B91" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C91">
         <v>1</v>
@@ -2984,7 +3136,7 @@
         <v>53</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -2992,7 +3144,7 @@
         <v>4</v>
       </c>
       <c r="B92" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C92">
         <v>1</v>
@@ -3001,7 +3153,7 @@
         <v>54</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -3009,7 +3161,7 @@
         <v>4</v>
       </c>
       <c r="B93" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C93">
         <v>1</v>
@@ -3018,7 +3170,7 @@
         <v>55</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -3026,7 +3178,7 @@
         <v>4</v>
       </c>
       <c r="B94" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C94">
         <v>1</v>
@@ -3035,7 +3187,7 @@
         <v>56</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="29.25">
@@ -3043,7 +3195,7 @@
         <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C95">
         <v>1</v>
@@ -3052,7 +3204,7 @@
         <v>57</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="29.25">
@@ -3060,7 +3212,7 @@
         <v>4</v>
       </c>
       <c r="B96" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C96">
         <v>1</v>
@@ -3069,7 +3221,7 @@
         <v>58</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="29.25">
@@ -3077,7 +3229,7 @@
         <v>4</v>
       </c>
       <c r="B97" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C97">
         <v>1</v>
@@ -3086,7 +3238,7 @@
         <v>59</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="29.25">
@@ -3094,7 +3246,7 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C98">
         <v>1</v>
@@ -3103,7 +3255,7 @@
         <v>60</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="29.25">
@@ -3111,7 +3263,7 @@
         <v>4</v>
       </c>
       <c r="B99" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -3120,7 +3272,7 @@
         <v>61</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="43.5">
@@ -3128,7 +3280,7 @@
         <v>4</v>
       </c>
       <c r="B100" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C100">
         <v>1</v>
@@ -3137,7 +3289,7 @@
         <v>62</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="29.25">
@@ -3145,7 +3297,7 @@
         <v>4</v>
       </c>
       <c r="B101" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C101">
         <v>1</v>
@@ -3154,7 +3306,7 @@
         <v>63</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="29.25">
@@ -3162,7 +3314,7 @@
         <v>4</v>
       </c>
       <c r="B102" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -3171,7 +3323,7 @@
         <v>64</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="29.25">
@@ -3179,7 +3331,7 @@
         <v>4</v>
       </c>
       <c r="B103" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C103">
         <v>1</v>
@@ -3188,7 +3340,7 @@
         <v>65</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="29.25">
@@ -3196,7 +3348,7 @@
         <v>4</v>
       </c>
       <c r="B104" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -3205,7 +3357,7 @@
         <v>66</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="29.25">
@@ -3213,7 +3365,7 @@
         <v>4</v>
       </c>
       <c r="B105" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C105">
         <v>1</v>
@@ -3222,7 +3374,7 @@
         <v>67</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="43.5">
@@ -3230,7 +3382,7 @@
         <v>4</v>
       </c>
       <c r="B106" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C106">
         <v>1</v>
@@ -3239,7 +3391,7 @@
         <v>68</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="43.5">
@@ -3247,7 +3399,7 @@
         <v>4</v>
       </c>
       <c r="B107" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C107">
         <v>1</v>
@@ -3256,7 +3408,7 @@
         <v>69</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="29.25">
@@ -3264,7 +3416,7 @@
         <v>4</v>
       </c>
       <c r="B108" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C108">
         <v>1</v>
@@ -3273,7 +3425,7 @@
         <v>70</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="109" spans="1:5" ht="57.75">
@@ -3281,7 +3433,7 @@
         <v>4</v>
       </c>
       <c r="B109" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C109">
         <v>1</v>
@@ -3290,7 +3442,7 @@
         <v>71</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="43.5">
@@ -3298,7 +3450,7 @@
         <v>4</v>
       </c>
       <c r="B110" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C110">
         <v>1</v>
@@ -3307,7 +3459,7 @@
         <v>72</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="29.25">
@@ -3315,7 +3467,7 @@
         <v>4</v>
       </c>
       <c r="B111" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C111">
         <v>1</v>
@@ -3324,7 +3476,7 @@
         <v>73</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="29.25">
@@ -3332,7 +3484,7 @@
         <v>4</v>
       </c>
       <c r="B112" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C112">
         <v>1</v>
@@ -3341,7 +3493,7 @@
         <v>74</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="29.25">
@@ -3349,7 +3501,7 @@
         <v>4</v>
       </c>
       <c r="B113" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C113">
         <v>1</v>
@@ -3358,7 +3510,7 @@
         <v>75</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="114" spans="1:5">

</xml_diff>